<commit_message>
Fix load profiles units and enable time-series convergence
</commit_message>
<xml_diff>
--- a/grodent-magnenat-mini-projet-trey/input-data/power_profile.xlsx
+++ b/grodent-magnenat-mini-projet-trey/input-data/power_profile.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\lutomasini\git\pandapower-heig-ui\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\max\github\rhtlab\grodent-magnenat-mini-projet-trey\input-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{353800EC-CB52-4900-9778-38AF3DA4C29F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BA03D21-B994-40C7-8217-E8E0DC244935}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{5FC146A3-AC37-46DC-AD92-E888F69598AC}"/>
+    <workbookView xWindow="686" yWindow="686" windowWidth="20983" windowHeight="14794" xr2:uid="{5FC146A3-AC37-46DC-AD92-E888F69598AC}"/>
   </bookViews>
   <sheets>
     <sheet name="load" sheetId="5" r:id="rId1"/>
@@ -130,9 +130,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office 2013 – 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -170,7 +170,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -276,7 +276,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -418,7 +418,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -427,14 +427,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB91AA0C-6E10-4C2C-B831-A2E20673E5F8}">
   <dimension ref="A1:BT98"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.3828125" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" style="1" customWidth="1"/>
-    <col min="2" max="23" width="12.7109375" style="4" customWidth="1"/>
-    <col min="24" max="39" width="12.7109375" customWidth="1"/>
+    <col min="1" max="1" width="11.3828125" style="1" customWidth="1"/>
+    <col min="2" max="23" width="12.69140625" style="4" customWidth="1"/>
+    <col min="24" max="39" width="12.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -515,7 +515,7 @@
       </c>
       <c r="AM1" s="6"/>
     </row>
-    <row r="2" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A2" s="7"/>
       <c r="B2" s="3" t="s">
         <v>1</v>
@@ -632,9 +632,15 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A3" s="1">
         <v>0</v>
+      </c>
+      <c r="B3" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C3" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N3" s="5"/>
       <c r="O3" s="5"/>
@@ -692,9 +698,15 @@
       <c r="BS3" s="4"/>
       <c r="BT3" s="4"/>
     </row>
-    <row r="4" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A4" s="1">
         <v>1.0416666666666666E-2</v>
+      </c>
+      <c r="B4" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C4" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N4" s="5"/>
       <c r="O4" s="5"/>
@@ -752,9 +764,15 @@
       <c r="BS4" s="4"/>
       <c r="BT4" s="4"/>
     </row>
-    <row r="5" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A5" s="1">
         <v>2.0833333333333301E-2</v>
+      </c>
+      <c r="B5" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C5" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N5" s="5"/>
       <c r="O5" s="5"/>
@@ -812,9 +830,15 @@
       <c r="BS5" s="4"/>
       <c r="BT5" s="4"/>
     </row>
-    <row r="6" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A6" s="1">
         <v>3.125E-2</v>
+      </c>
+      <c r="B6" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C6" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N6" s="5"/>
       <c r="O6" s="5"/>
@@ -872,9 +896,15 @@
       <c r="BS6" s="4"/>
       <c r="BT6" s="4"/>
     </row>
-    <row r="7" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A7" s="1">
         <v>4.1666666666666699E-2</v>
+      </c>
+      <c r="B7" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C7" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N7" s="5"/>
       <c r="O7" s="5"/>
@@ -932,9 +962,15 @@
       <c r="BS7" s="4"/>
       <c r="BT7" s="4"/>
     </row>
-    <row r="8" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A8" s="1">
         <v>5.2083333333333301E-2</v>
+      </c>
+      <c r="B8" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C8" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N8" s="5"/>
       <c r="O8" s="5"/>
@@ -992,9 +1028,15 @@
       <c r="BS8" s="4"/>
       <c r="BT8" s="4"/>
     </row>
-    <row r="9" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A9" s="1">
         <v>6.25E-2</v>
+      </c>
+      <c r="B9" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C9" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N9" s="5"/>
       <c r="O9" s="5"/>
@@ -1052,9 +1094,15 @@
       <c r="BS9" s="4"/>
       <c r="BT9" s="4"/>
     </row>
-    <row r="10" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A10" s="1">
         <v>7.2916666666666699E-2</v>
+      </c>
+      <c r="B10" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C10" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N10" s="5"/>
       <c r="O10" s="5"/>
@@ -1112,9 +1160,15 @@
       <c r="BS10" s="4"/>
       <c r="BT10" s="4"/>
     </row>
-    <row r="11" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A11" s="1">
         <v>8.3333333333333301E-2</v>
+      </c>
+      <c r="B11" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C11" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N11" s="5"/>
       <c r="O11" s="5"/>
@@ -1172,9 +1226,15 @@
       <c r="BS11" s="4"/>
       <c r="BT11" s="4"/>
     </row>
-    <row r="12" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A12" s="1">
         <v>9.375E-2</v>
+      </c>
+      <c r="B12" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C12" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N12" s="5"/>
       <c r="O12" s="5"/>
@@ -1232,9 +1292,15 @@
       <c r="BS12" s="4"/>
       <c r="BT12" s="4"/>
     </row>
-    <row r="13" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A13" s="1">
         <v>0.104166666666667</v>
+      </c>
+      <c r="B13" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C13" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N13" s="5"/>
       <c r="O13" s="5"/>
@@ -1292,9 +1358,15 @@
       <c r="BS13" s="4"/>
       <c r="BT13" s="4"/>
     </row>
-    <row r="14" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A14" s="1">
         <v>0.114583333333333</v>
+      </c>
+      <c r="B14" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C14" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N14" s="5"/>
       <c r="O14" s="5"/>
@@ -1352,9 +1424,15 @@
       <c r="BS14" s="4"/>
       <c r="BT14" s="4"/>
     </row>
-    <row r="15" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A15" s="1">
         <v>0.125</v>
+      </c>
+      <c r="B15" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C15" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N15" s="5"/>
       <c r="O15" s="5"/>
@@ -1412,9 +1490,15 @@
       <c r="BS15" s="4"/>
       <c r="BT15" s="4"/>
     </row>
-    <row r="16" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A16" s="1">
         <v>0.13541666666666699</v>
+      </c>
+      <c r="B16" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C16" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N16" s="5"/>
       <c r="O16" s="5"/>
@@ -1472,9 +1556,15 @@
       <c r="BS16" s="4"/>
       <c r="BT16" s="4"/>
     </row>
-    <row r="17" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A17" s="1">
         <v>0.14583333333333301</v>
+      </c>
+      <c r="B17" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C17" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N17" s="5"/>
       <c r="O17" s="5"/>
@@ -1532,9 +1622,15 @@
       <c r="BS17" s="4"/>
       <c r="BT17" s="4"/>
     </row>
-    <row r="18" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A18" s="1">
         <v>0.15625</v>
+      </c>
+      <c r="B18" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C18" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N18" s="5"/>
       <c r="O18" s="5"/>
@@ -1592,9 +1688,15 @@
       <c r="BS18" s="4"/>
       <c r="BT18" s="4"/>
     </row>
-    <row r="19" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A19" s="1">
         <v>0.16666666666666699</v>
+      </c>
+      <c r="B19" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C19" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N19" s="5"/>
       <c r="O19" s="5"/>
@@ -1652,9 +1754,15 @@
       <c r="BS19" s="4"/>
       <c r="BT19" s="4"/>
     </row>
-    <row r="20" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A20" s="1">
         <v>0.17708333333333301</v>
+      </c>
+      <c r="B20" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C20" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N20" s="5"/>
       <c r="O20" s="5"/>
@@ -1712,9 +1820,15 @@
       <c r="BS20" s="4"/>
       <c r="BT20" s="4"/>
     </row>
-    <row r="21" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A21" s="1">
         <v>0.1875</v>
+      </c>
+      <c r="B21" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C21" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N21" s="5"/>
       <c r="O21" s="5"/>
@@ -1772,9 +1886,15 @@
       <c r="BS21" s="4"/>
       <c r="BT21" s="4"/>
     </row>
-    <row r="22" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A22" s="1">
         <v>0.19791666666666699</v>
+      </c>
+      <c r="B22" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C22" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N22" s="5"/>
       <c r="O22" s="5"/>
@@ -1832,9 +1952,15 @@
       <c r="BS22" s="4"/>
       <c r="BT22" s="4"/>
     </row>
-    <row r="23" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A23" s="1">
         <v>0.20833333333333301</v>
+      </c>
+      <c r="B23" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C23" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N23" s="5"/>
       <c r="O23" s="5"/>
@@ -1892,9 +2018,15 @@
       <c r="BS23" s="4"/>
       <c r="BT23" s="4"/>
     </row>
-    <row r="24" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A24" s="1">
         <v>0.21875</v>
+      </c>
+      <c r="B24" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C24" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N24" s="5"/>
       <c r="O24" s="5"/>
@@ -1952,9 +2084,15 @@
       <c r="BS24" s="4"/>
       <c r="BT24" s="4"/>
     </row>
-    <row r="25" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A25" s="1">
         <v>0.22916666666666699</v>
+      </c>
+      <c r="B25" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C25" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N25" s="5"/>
       <c r="O25" s="5"/>
@@ -2012,9 +2150,15 @@
       <c r="BS25" s="4"/>
       <c r="BT25" s="4"/>
     </row>
-    <row r="26" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A26" s="1">
         <v>0.23958333333333301</v>
+      </c>
+      <c r="B26" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C26" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N26" s="5"/>
       <c r="O26" s="5"/>
@@ -2072,9 +2216,15 @@
       <c r="BS26" s="4"/>
       <c r="BT26" s="4"/>
     </row>
-    <row r="27" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A27" s="1">
         <v>0.25</v>
+      </c>
+      <c r="B27" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C27" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N27" s="5"/>
       <c r="O27" s="5"/>
@@ -2132,9 +2282,15 @@
       <c r="BS27" s="4"/>
       <c r="BT27" s="4"/>
     </row>
-    <row r="28" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A28" s="1">
         <v>0.26041666666666702</v>
+      </c>
+      <c r="B28" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C28" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N28" s="5"/>
       <c r="O28" s="5"/>
@@ -2192,9 +2348,15 @@
       <c r="BS28" s="4"/>
       <c r="BT28" s="4"/>
     </row>
-    <row r="29" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A29" s="1">
         <v>0.27083333333333298</v>
+      </c>
+      <c r="B29" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C29" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N29" s="5"/>
       <c r="O29" s="5"/>
@@ -2252,9 +2414,15 @@
       <c r="BS29" s="4"/>
       <c r="BT29" s="4"/>
     </row>
-    <row r="30" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A30" s="1">
         <v>0.28125</v>
+      </c>
+      <c r="B30" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C30" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N30" s="5"/>
       <c r="O30" s="5"/>
@@ -2312,9 +2480,15 @@
       <c r="BS30" s="4"/>
       <c r="BT30" s="4"/>
     </row>
-    <row r="31" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A31" s="1">
         <v>0.29166666666666702</v>
+      </c>
+      <c r="B31" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C31" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N31" s="5"/>
       <c r="O31" s="5"/>
@@ -2372,9 +2546,15 @@
       <c r="BS31" s="4"/>
       <c r="BT31" s="4"/>
     </row>
-    <row r="32" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A32" s="1">
         <v>0.30208333333333298</v>
+      </c>
+      <c r="B32" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C32" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N32" s="5"/>
       <c r="O32" s="5"/>
@@ -2432,9 +2612,15 @@
       <c r="BS32" s="4"/>
       <c r="BT32" s="4"/>
     </row>
-    <row r="33" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A33" s="1">
         <v>0.3125</v>
+      </c>
+      <c r="B33" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C33" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N33" s="5"/>
       <c r="O33" s="5"/>
@@ -2492,9 +2678,15 @@
       <c r="BS33" s="4"/>
       <c r="BT33" s="4"/>
     </row>
-    <row r="34" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A34" s="1">
         <v>0.32291666666666702</v>
+      </c>
+      <c r="B34" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C34" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N34" s="5"/>
       <c r="O34" s="5"/>
@@ -2552,9 +2744,15 @@
       <c r="BS34" s="4"/>
       <c r="BT34" s="4"/>
     </row>
-    <row r="35" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A35" s="1">
         <v>0.33333333333333298</v>
+      </c>
+      <c r="B35" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C35" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N35" s="5"/>
       <c r="O35" s="5"/>
@@ -2612,9 +2810,15 @@
       <c r="BS35" s="4"/>
       <c r="BT35" s="4"/>
     </row>
-    <row r="36" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A36" s="1">
         <v>0.34375</v>
+      </c>
+      <c r="B36" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C36" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N36" s="5"/>
       <c r="O36" s="5"/>
@@ -2672,9 +2876,15 @@
       <c r="BS36" s="4"/>
       <c r="BT36" s="4"/>
     </row>
-    <row r="37" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A37" s="1">
         <v>0.35416666666666702</v>
+      </c>
+      <c r="B37" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C37" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N37" s="5"/>
       <c r="O37" s="5"/>
@@ -2732,9 +2942,15 @@
       <c r="BS37" s="4"/>
       <c r="BT37" s="4"/>
     </row>
-    <row r="38" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A38" s="1">
         <v>0.36458333333333298</v>
+      </c>
+      <c r="B38" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C38" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N38" s="5"/>
       <c r="O38" s="5"/>
@@ -2792,9 +3008,15 @@
       <c r="BS38" s="4"/>
       <c r="BT38" s="4"/>
     </row>
-    <row r="39" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A39" s="1">
         <v>0.375</v>
+      </c>
+      <c r="B39" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C39" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N39" s="5"/>
       <c r="O39" s="5"/>
@@ -2852,9 +3074,15 @@
       <c r="BS39" s="4"/>
       <c r="BT39" s="4"/>
     </row>
-    <row r="40" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A40" s="1">
         <v>0.38541666666666702</v>
+      </c>
+      <c r="B40" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C40" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N40" s="5"/>
       <c r="O40" s="5"/>
@@ -2912,9 +3140,15 @@
       <c r="BS40" s="4"/>
       <c r="BT40" s="4"/>
     </row>
-    <row r="41" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A41" s="1">
         <v>0.39583333333333298</v>
+      </c>
+      <c r="B41" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C41" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N41" s="5"/>
       <c r="O41" s="5"/>
@@ -2972,9 +3206,15 @@
       <c r="BS41" s="4"/>
       <c r="BT41" s="4"/>
     </row>
-    <row r="42" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A42" s="1">
         <v>0.40625</v>
+      </c>
+      <c r="B42" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C42" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N42" s="5"/>
       <c r="O42" s="5"/>
@@ -3032,9 +3272,15 @@
       <c r="BS42" s="4"/>
       <c r="BT42" s="4"/>
     </row>
-    <row r="43" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A43" s="1">
         <v>0.41666666666666702</v>
+      </c>
+      <c r="B43" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C43" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N43" s="5"/>
       <c r="O43" s="5"/>
@@ -3092,9 +3338,15 @@
       <c r="BS43" s="4"/>
       <c r="BT43" s="4"/>
     </row>
-    <row r="44" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A44" s="1">
         <v>0.42708333333333298</v>
+      </c>
+      <c r="B44" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C44" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N44" s="5"/>
       <c r="O44" s="5"/>
@@ -3152,9 +3404,15 @@
       <c r="BS44" s="4"/>
       <c r="BT44" s="4"/>
     </row>
-    <row r="45" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A45" s="1">
         <v>0.4375</v>
+      </c>
+      <c r="B45" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C45" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N45" s="5"/>
       <c r="O45" s="5"/>
@@ -3212,9 +3470,15 @@
       <c r="BS45" s="4"/>
       <c r="BT45" s="4"/>
     </row>
-    <row r="46" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A46" s="1">
         <v>0.44791666666666702</v>
+      </c>
+      <c r="B46" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C46" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N46" s="5"/>
       <c r="O46" s="5"/>
@@ -3272,9 +3536,15 @@
       <c r="BS46" s="4"/>
       <c r="BT46" s="4"/>
     </row>
-    <row r="47" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A47" s="1">
         <v>0.45833333333333298</v>
+      </c>
+      <c r="B47" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C47" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N47" s="5"/>
       <c r="O47" s="5"/>
@@ -3332,9 +3602,15 @@
       <c r="BS47" s="4"/>
       <c r="BT47" s="4"/>
     </row>
-    <row r="48" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A48" s="1">
         <v>0.46875</v>
+      </c>
+      <c r="B48" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C48" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N48" s="5"/>
       <c r="O48" s="5"/>
@@ -3392,9 +3668,15 @@
       <c r="BS48" s="4"/>
       <c r="BT48" s="4"/>
     </row>
-    <row r="49" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A49" s="1">
         <v>0.47916666666666702</v>
+      </c>
+      <c r="B49" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C49" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N49" s="5"/>
       <c r="O49" s="5"/>
@@ -3452,9 +3734,15 @@
       <c r="BS49" s="4"/>
       <c r="BT49" s="4"/>
     </row>
-    <row r="50" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A50" s="1">
         <v>0.48958333333333298</v>
+      </c>
+      <c r="B50" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C50" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N50" s="5"/>
       <c r="O50" s="5"/>
@@ -3512,9 +3800,15 @@
       <c r="BS50" s="4"/>
       <c r="BT50" s="4"/>
     </row>
-    <row r="51" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A51" s="1">
         <v>0.5</v>
+      </c>
+      <c r="B51" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C51" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N51" s="5"/>
       <c r="O51" s="5"/>
@@ -3572,9 +3866,15 @@
       <c r="BS51" s="4"/>
       <c r="BT51" s="4"/>
     </row>
-    <row r="52" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A52" s="1">
         <v>0.51041666666666696</v>
+      </c>
+      <c r="B52" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C52" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N52" s="5"/>
       <c r="O52" s="5"/>
@@ -3632,9 +3932,15 @@
       <c r="BS52" s="4"/>
       <c r="BT52" s="4"/>
     </row>
-    <row r="53" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A53" s="1">
         <v>0.52083333333333304</v>
+      </c>
+      <c r="B53" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C53" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N53" s="5"/>
       <c r="O53" s="5"/>
@@ -3692,9 +3998,15 @@
       <c r="BS53" s="4"/>
       <c r="BT53" s="4"/>
     </row>
-    <row r="54" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A54" s="1">
         <v>0.53125</v>
+      </c>
+      <c r="B54" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C54" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N54" s="5"/>
       <c r="O54" s="5"/>
@@ -3752,9 +4064,15 @@
       <c r="BS54" s="4"/>
       <c r="BT54" s="4"/>
     </row>
-    <row r="55" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A55" s="1">
         <v>0.54166666666666696</v>
+      </c>
+      <c r="B55" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C55" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N55" s="5"/>
       <c r="O55" s="5"/>
@@ -3812,9 +4130,15 @@
       <c r="BS55" s="4"/>
       <c r="BT55" s="4"/>
     </row>
-    <row r="56" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A56" s="1">
         <v>0.55208333333333304</v>
+      </c>
+      <c r="B56" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C56" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N56" s="5"/>
       <c r="O56" s="5"/>
@@ -3872,9 +4196,15 @@
       <c r="BS56" s="4"/>
       <c r="BT56" s="4"/>
     </row>
-    <row r="57" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A57" s="1">
         <v>0.5625</v>
+      </c>
+      <c r="B57" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C57" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N57" s="5"/>
       <c r="O57" s="5"/>
@@ -3932,9 +4262,15 @@
       <c r="BS57" s="4"/>
       <c r="BT57" s="4"/>
     </row>
-    <row r="58" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A58" s="1">
         <v>0.57291666666666696</v>
+      </c>
+      <c r="B58" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C58" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N58" s="5"/>
       <c r="O58" s="5"/>
@@ -3992,9 +4328,15 @@
       <c r="BS58" s="4"/>
       <c r="BT58" s="4"/>
     </row>
-    <row r="59" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A59" s="1">
         <v>0.58333333333333304</v>
+      </c>
+      <c r="B59" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C59" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N59" s="5"/>
       <c r="O59" s="5"/>
@@ -4052,9 +4394,15 @@
       <c r="BS59" s="4"/>
       <c r="BT59" s="4"/>
     </row>
-    <row r="60" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A60" s="1">
         <v>0.59375</v>
+      </c>
+      <c r="B60" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C60" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N60" s="5"/>
       <c r="O60" s="5"/>
@@ -4112,9 +4460,15 @@
       <c r="BS60" s="4"/>
       <c r="BT60" s="4"/>
     </row>
-    <row r="61" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A61" s="1">
         <v>0.60416666666666696</v>
+      </c>
+      <c r="B61" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C61" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N61" s="5"/>
       <c r="O61" s="5"/>
@@ -4172,9 +4526,15 @@
       <c r="BS61" s="4"/>
       <c r="BT61" s="4"/>
     </row>
-    <row r="62" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A62" s="1">
         <v>0.61458333333333304</v>
+      </c>
+      <c r="B62" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C62" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N62" s="5"/>
       <c r="O62" s="5"/>
@@ -4232,9 +4592,15 @@
       <c r="BS62" s="4"/>
       <c r="BT62" s="4"/>
     </row>
-    <row r="63" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A63" s="1">
         <v>0.625</v>
+      </c>
+      <c r="B63" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C63" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N63" s="5"/>
       <c r="O63" s="5"/>
@@ -4292,9 +4658,15 @@
       <c r="BS63" s="4"/>
       <c r="BT63" s="4"/>
     </row>
-    <row r="64" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A64" s="1">
         <v>0.63541666666666696</v>
+      </c>
+      <c r="B64" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C64" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N64" s="5"/>
       <c r="O64" s="5"/>
@@ -4352,9 +4724,15 @@
       <c r="BS64" s="4"/>
       <c r="BT64" s="4"/>
     </row>
-    <row r="65" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A65" s="1">
         <v>0.64583333333333304</v>
+      </c>
+      <c r="B65" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C65" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N65" s="5"/>
       <c r="O65" s="5"/>
@@ -4412,9 +4790,15 @@
       <c r="BS65" s="4"/>
       <c r="BT65" s="4"/>
     </row>
-    <row r="66" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A66" s="1">
         <v>0.65625</v>
+      </c>
+      <c r="B66" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C66" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N66" s="5"/>
       <c r="O66" s="5"/>
@@ -4472,9 +4856,15 @@
       <c r="BS66" s="4"/>
       <c r="BT66" s="4"/>
     </row>
-    <row r="67" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A67" s="1">
         <v>0.66666666666666696</v>
+      </c>
+      <c r="B67" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C67" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N67" s="5"/>
       <c r="O67" s="5"/>
@@ -4532,9 +4922,15 @@
       <c r="BS67" s="4"/>
       <c r="BT67" s="4"/>
     </row>
-    <row r="68" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A68" s="1">
         <v>0.67708333333333304</v>
+      </c>
+      <c r="B68" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C68" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N68" s="5"/>
       <c r="O68" s="5"/>
@@ -4592,9 +4988,15 @@
       <c r="BS68" s="4"/>
       <c r="BT68" s="4"/>
     </row>
-    <row r="69" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A69" s="1">
         <v>0.6875</v>
+      </c>
+      <c r="B69" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C69" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N69" s="5"/>
       <c r="O69" s="5"/>
@@ -4652,9 +5054,15 @@
       <c r="BS69" s="4"/>
       <c r="BT69" s="4"/>
     </row>
-    <row r="70" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A70" s="1">
         <v>0.69791666666666696</v>
+      </c>
+      <c r="B70" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C70" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N70" s="5"/>
       <c r="O70" s="5"/>
@@ -4712,9 +5120,15 @@
       <c r="BS70" s="4"/>
       <c r="BT70" s="4"/>
     </row>
-    <row r="71" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A71" s="1">
         <v>0.70833333333333304</v>
+      </c>
+      <c r="B71" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C71" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N71" s="5"/>
       <c r="O71" s="5"/>
@@ -4772,9 +5186,15 @@
       <c r="BS71" s="4"/>
       <c r="BT71" s="4"/>
     </row>
-    <row r="72" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A72" s="1">
         <v>0.71875</v>
+      </c>
+      <c r="B72" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C72" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N72" s="5"/>
       <c r="O72" s="5"/>
@@ -4832,9 +5252,15 @@
       <c r="BS72" s="4"/>
       <c r="BT72" s="4"/>
     </row>
-    <row r="73" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A73" s="1">
         <v>0.72916666666666696</v>
+      </c>
+      <c r="B73" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C73" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N73" s="5"/>
       <c r="O73" s="5"/>
@@ -4892,9 +5318,15 @@
       <c r="BS73" s="4"/>
       <c r="BT73" s="4"/>
     </row>
-    <row r="74" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A74" s="1">
         <v>0.73958333333333304</v>
+      </c>
+      <c r="B74" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C74" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N74" s="5"/>
       <c r="O74" s="5"/>
@@ -4952,9 +5384,15 @@
       <c r="BS74" s="4"/>
       <c r="BT74" s="4"/>
     </row>
-    <row r="75" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A75" s="1">
         <v>0.75</v>
+      </c>
+      <c r="B75" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C75" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N75" s="5"/>
       <c r="O75" s="5"/>
@@ -5012,9 +5450,15 @@
       <c r="BS75" s="4"/>
       <c r="BT75" s="4"/>
     </row>
-    <row r="76" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A76" s="1">
         <v>0.76041666666666696</v>
+      </c>
+      <c r="B76" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C76" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N76" s="5"/>
       <c r="O76" s="5"/>
@@ -5072,9 +5516,15 @@
       <c r="BS76" s="4"/>
       <c r="BT76" s="4"/>
     </row>
-    <row r="77" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A77" s="1">
         <v>0.77083333333333304</v>
+      </c>
+      <c r="B77" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C77" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N77" s="5"/>
       <c r="O77" s="5"/>
@@ -5132,9 +5582,15 @@
       <c r="BS77" s="4"/>
       <c r="BT77" s="4"/>
     </row>
-    <row r="78" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A78" s="1">
         <v>0.78125</v>
+      </c>
+      <c r="B78" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C78" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N78" s="5"/>
       <c r="O78" s="5"/>
@@ -5192,9 +5648,15 @@
       <c r="BS78" s="4"/>
       <c r="BT78" s="4"/>
     </row>
-    <row r="79" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A79" s="1">
         <v>0.79166666666666696</v>
+      </c>
+      <c r="B79" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C79" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N79" s="5"/>
       <c r="O79" s="5"/>
@@ -5252,9 +5714,15 @@
       <c r="BS79" s="4"/>
       <c r="BT79" s="4"/>
     </row>
-    <row r="80" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A80" s="1">
         <v>0.80208333333333304</v>
+      </c>
+      <c r="B80" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C80" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N80" s="5"/>
       <c r="O80" s="5"/>
@@ -5312,9 +5780,15 @@
       <c r="BS80" s="4"/>
       <c r="BT80" s="4"/>
     </row>
-    <row r="81" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A81" s="1">
         <v>0.8125</v>
+      </c>
+      <c r="B81" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C81" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N81" s="5"/>
       <c r="O81" s="5"/>
@@ -5372,9 +5846,15 @@
       <c r="BS81" s="4"/>
       <c r="BT81" s="4"/>
     </row>
-    <row r="82" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A82" s="1">
         <v>0.82291666666666696</v>
+      </c>
+      <c r="B82" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C82" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N82" s="5"/>
       <c r="O82" s="5"/>
@@ -5432,9 +5912,15 @@
       <c r="BS82" s="4"/>
       <c r="BT82" s="4"/>
     </row>
-    <row r="83" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A83" s="1">
         <v>0.83333333333333304</v>
+      </c>
+      <c r="B83" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C83" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N83" s="5"/>
       <c r="O83" s="5"/>
@@ -5492,9 +5978,15 @@
       <c r="BS83" s="4"/>
       <c r="BT83" s="4"/>
     </row>
-    <row r="84" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A84" s="1">
         <v>0.84375</v>
+      </c>
+      <c r="B84" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C84" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N84" s="5"/>
       <c r="O84" s="5"/>
@@ -5552,9 +6044,15 @@
       <c r="BS84" s="4"/>
       <c r="BT84" s="4"/>
     </row>
-    <row r="85" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A85" s="1">
         <v>0.85416666666666696</v>
+      </c>
+      <c r="B85" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C85" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N85" s="5"/>
       <c r="O85" s="5"/>
@@ -5612,9 +6110,15 @@
       <c r="BS85" s="4"/>
       <c r="BT85" s="4"/>
     </row>
-    <row r="86" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A86" s="1">
         <v>0.86458333333333304</v>
+      </c>
+      <c r="B86" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C86" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N86" s="5"/>
       <c r="O86" s="5"/>
@@ -5672,9 +6176,15 @@
       <c r="BS86" s="4"/>
       <c r="BT86" s="4"/>
     </row>
-    <row r="87" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A87" s="1">
         <v>0.875</v>
+      </c>
+      <c r="B87" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C87" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N87" s="5"/>
       <c r="O87" s="5"/>
@@ -5732,9 +6242,15 @@
       <c r="BS87" s="4"/>
       <c r="BT87" s="4"/>
     </row>
-    <row r="88" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A88" s="1">
         <v>0.88541666666666696</v>
+      </c>
+      <c r="B88" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C88" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N88" s="5"/>
       <c r="O88" s="5"/>
@@ -5792,9 +6308,15 @@
       <c r="BS88" s="4"/>
       <c r="BT88" s="4"/>
     </row>
-    <row r="89" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A89" s="1">
         <v>0.89583333333333304</v>
+      </c>
+      <c r="B89" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C89" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N89" s="5"/>
       <c r="O89" s="5"/>
@@ -5852,9 +6374,15 @@
       <c r="BS89" s="4"/>
       <c r="BT89" s="4"/>
     </row>
-    <row r="90" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A90" s="1">
         <v>0.90625</v>
+      </c>
+      <c r="B90" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C90" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N90" s="5"/>
       <c r="O90" s="5"/>
@@ -5912,9 +6440,15 @@
       <c r="BS90" s="4"/>
       <c r="BT90" s="4"/>
     </row>
-    <row r="91" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A91" s="1">
         <v>0.91666666666666696</v>
+      </c>
+      <c r="B91" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C91" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N91" s="5"/>
       <c r="O91" s="5"/>
@@ -5972,9 +6506,15 @@
       <c r="BS91" s="4"/>
       <c r="BT91" s="4"/>
     </row>
-    <row r="92" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A92" s="1">
         <v>0.92708333333333304</v>
+      </c>
+      <c r="B92" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C92" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N92" s="5"/>
       <c r="O92" s="5"/>
@@ -6032,9 +6572,15 @@
       <c r="BS92" s="4"/>
       <c r="BT92" s="4"/>
     </row>
-    <row r="93" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A93" s="1">
         <v>0.9375</v>
+      </c>
+      <c r="B93" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C93" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N93" s="5"/>
       <c r="O93" s="5"/>
@@ -6092,9 +6638,15 @@
       <c r="BS93" s="4"/>
       <c r="BT93" s="4"/>
     </row>
-    <row r="94" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A94" s="1">
         <v>0.94791666666666696</v>
+      </c>
+      <c r="B94" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C94" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N94" s="5"/>
       <c r="O94" s="5"/>
@@ -6152,9 +6704,15 @@
       <c r="BS94" s="4"/>
       <c r="BT94" s="4"/>
     </row>
-    <row r="95" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A95" s="1">
         <v>0.95833333333333304</v>
+      </c>
+      <c r="B95" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C95" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N95" s="5"/>
       <c r="O95" s="5"/>
@@ -6212,9 +6770,15 @@
       <c r="BS95" s="4"/>
       <c r="BT95" s="4"/>
     </row>
-    <row r="96" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A96" s="1">
         <v>0.96875</v>
+      </c>
+      <c r="B96" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C96" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N96" s="5"/>
       <c r="O96" s="5"/>
@@ -6272,9 +6836,15 @@
       <c r="BS96" s="4"/>
       <c r="BT96" s="4"/>
     </row>
-    <row r="97" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A97" s="1">
         <v>0.97916666666666696</v>
+      </c>
+      <c r="B97" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C97" s="4">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="N97" s="5"/>
       <c r="O97" s="5"/>
@@ -6332,14 +6902,20 @@
       <c r="BS97" s="4"/>
       <c r="BT97" s="4"/>
     </row>
-    <row r="98" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:72" x14ac:dyDescent="0.4">
       <c r="A98" s="1">
         <v>0.98958333333333304</v>
       </c>
+      <c r="B98" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="C98" s="4">
+        <v>5.0000000000000001E-3</v>
+      </c>
     </row>
   </sheetData>
   <protectedRanges>
-    <protectedRange sqref="B4:B97 B3:G3 C4:G98" name="Plage1_1_1"/>
+    <protectedRange sqref="B3:G98" name="Plage1_1_1"/>
     <protectedRange sqref="H3:I3 H4:H97 I4:I98" name="Plage1_5"/>
     <protectedRange sqref="J3:K3 K4:K97 J4:J98" name="Plage1_6"/>
     <protectedRange sqref="L3:M97" name="Plage1_8"/>
@@ -6377,13 +6953,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB0724F9-1790-4ECA-B4EA-D773CFA5B42B}">
   <dimension ref="A1:AM26"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.3828125" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" style="1" customWidth="1"/>
-    <col min="2" max="39" width="12.7109375" customWidth="1"/>
+    <col min="1" max="1" width="11.3828125" style="1" customWidth="1"/>
+    <col min="2" max="39" width="12.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -6464,7 +7040,7 @@
       </c>
       <c r="AM1" s="8"/>
     </row>
-    <row r="2" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A2" s="7"/>
       <c r="B2" s="2" t="s">
         <v>1</v>
@@ -6581,122 +7157,122 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A3" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A4" s="1">
         <v>4.1666666666666664E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A5" s="1">
         <v>8.3333333333333301E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A6" s="1">
         <v>0.125</v>
       </c>
     </row>
-    <row r="7" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A7" s="1">
         <v>0.16666666666666699</v>
       </c>
     </row>
-    <row r="8" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A8" s="1">
         <v>0.20833333333333301</v>
       </c>
     </row>
-    <row r="9" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A9" s="1">
         <v>0.25</v>
       </c>
     </row>
-    <row r="10" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A10" s="1">
         <v>0.29166666666666702</v>
       </c>
     </row>
-    <row r="11" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A11" s="1">
         <v>0.33333333333333298</v>
       </c>
     </row>
-    <row r="12" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A12" s="1">
         <v>0.375</v>
       </c>
     </row>
-    <row r="13" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A13" s="1">
         <v>0.41666666666666702</v>
       </c>
     </row>
-    <row r="14" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A14" s="1">
         <v>0.45833333333333298</v>
       </c>
     </row>
-    <row r="15" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A15" s="1">
         <v>0.5</v>
       </c>
     </row>
-    <row r="16" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A16" s="1">
         <v>0.54166666666666696</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A17" s="1">
         <v>0.58333333333333304</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A18" s="1">
         <v>0.625</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A19" s="1">
         <v>0.66666666666666696</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A20" s="1">
         <v>0.70833333333333304</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A21" s="1">
         <v>0.75</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A22" s="1">
         <v>0.79166666666666696</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A23" s="1">
         <v>0.83333333333333304</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A24" s="1">
         <v>0.875</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A25" s="1">
         <v>0.91666666666666696</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A26" s="1">
         <v>0.95833333333333304</v>
       </c>

</xml_diff>